<commit_message>
docs: UC-07 workbook workflow refreshed — template fill and placeholder guard as steps 1-2
Sheet 3 grows from 19 to 21 steps: the customer filling 00-TEMPLATE and the
unfilled-placeholder guard now open the workflow, with renumbering and the
journey-strip mirror noted. Sheet 9 gains the template row (refused while
unfilled, ~15 min to complete).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4JExjQdDmtQgo57VcSgGB
</commit_message>
<xml_diff>
--- a/usecases/uc-07-doc-driven-deployment/TCS-Agentic-AI-UC07-Doc-Driven-Deployment.xlsx
+++ b/usecases/uc-07-doc-driven-deployment/TCS-Agentic-AI-UC07-Doc-Driven-Deployment.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="280">
   <si>
     <t>TCS Agentic AI — Document-Driven Application Deployment  ·  UC-07</t>
   </si>
@@ -162,7 +162,7 @@
     <t>End-to-end workflow — every step, with its actor</t>
   </si>
   <si>
-    <t>14 automatic · 2 AI · 3 human · ends at a URL a person can click</t>
+    <t>15 automatic · 2 AI · 4 human · ends at a URL a person can click</t>
   </si>
   <si>
     <t>#</t>
@@ -174,10 +174,22 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Requirement document authored and PR-reviewed in Git</t>
-  </si>
-  <si>
-    <t>Markdown or Word; the tables are the contract, the prose is documentation</t>
+    <t>Customer fills the requirement TEMPLATE</t>
+  </si>
+  <si>
+    <t>00-TEMPLATE .md/.docx — guided three-tier scaffold; every decision is a placeholder in double angle brackets, working defaults everywhere else, guidance prose beside each field, field-reference appendix</t>
+  </si>
+  <si>
+    <t>Unfilled-placeholder guard</t>
+  </si>
+  <si>
+    <t>Generation REFUSES while any placeholder remains and names the missing fields — a half-filled template can never reach a cluster</t>
+  </si>
+  <si>
+    <t>Document authored / PR-reviewed in Git</t>
+  </si>
+  <si>
+    <t>Markdown or Word; the tables are the contract, the prose is documentation. Boutique doc = the completed example of the same template</t>
   </si>
   <si>
     <t>Document loaded — upload, paste, or 'Load from Git'</t>
@@ -288,7 +300,7 @@
     <t>UC-05 machinery reasons over logs, events and probes; proposes a fix a human approves (auto-wiring is roadmap)</t>
   </si>
   <si>
-    <t>Steps 7, 10 and 18 are the only places a person is required — review, deploy, and the final click that proves it works.</t>
+    <t>Steps 1, 9, 12 and 20 are the only places a person is required — fill the template, review, deploy, and the final click that proves it works. The console mirrors this as a live journey strip: Document ▸ Generate ▸ Review+checks ▸ Dry-run ▸ Deploy ▸ Verify ▸ Open app.</t>
   </si>
   <si>
     <t>Where the agentic AI actually is — an honest map</t>
@@ -607,6 +619,15 @@
   </si>
   <si>
     <t>Expected result</t>
+  </si>
+  <si>
+    <t>00-TEMPLATE (customer-facing)</t>
+  </si>
+  <si>
+    <t>The fill-in-the-blanks scaffold: three tiers, guided placeholders, field-reference appendix. Generation refuses until every placeholder is filled — and names the missing ones</t>
+  </si>
+  <si>
+    <t>Refused while unfilled; ~15 min to complete</t>
   </si>
   <si>
     <t>01-hello-web</t>
@@ -847,7 +868,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -942,6 +963,11 @@
       <b/>
       <color rgb="FF155E75"/>
       <sz val="10.5"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF92400E"/>
+      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1056,7 +1082,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1109,13 +1135,16 @@
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -1606,17 +1635,17 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
@@ -1624,68 +1653,68 @@
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>212</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>213</v>
+        <v>218</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>216</v>
+        <v>221</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>219</v>
+        <v>224</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>221</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>222</v>
+        <v>227</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>224</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>225</v>
+        <v>230</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>228</v>
+        <v>233</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -1712,80 +1741,80 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
@@ -1815,124 +1844,124 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>41</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>41</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>41</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>41</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>41</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
@@ -2052,7 +2081,7 @@
   <sheetPr>
     <tabColor rgb="FF2563EB"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2112,8 +2141,8 @@
       <c r="B6" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>38</v>
+      <c r="C6" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>53</v>
@@ -2126,8 +2155,8 @@
       <c r="B7" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>35</v>
+      <c r="C7" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>55</v>
@@ -2140,8 +2169,8 @@
       <c r="B8" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>35</v>
+      <c r="C8" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>57</v>
@@ -2154,8 +2183,8 @@
       <c r="B9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>32</v>
+      <c r="C9" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>59</v>
@@ -2182,8 +2211,8 @@
       <c r="B11" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>38</v>
+      <c r="C11" s="9" t="s">
+        <v>32</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>63</v>
@@ -2210,8 +2239,8 @@
       <c r="B13" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>35</v>
+      <c r="C13" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>67</v>
@@ -2224,8 +2253,8 @@
       <c r="B14" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>38</v>
+      <c r="C14" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>69</v>
@@ -2252,8 +2281,8 @@
       <c r="B16" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>35</v>
+      <c r="C16" s="11" t="s">
+        <v>38</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>73</v>
@@ -2336,8 +2365,8 @@
       <c r="B22" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C22" s="11" t="s">
-        <v>38</v>
+      <c r="C22" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>85</v>
@@ -2350,26 +2379,54 @@
       <c r="B23" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>32</v>
+      <c r="C23" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="24" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
+    <row r="24" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="7">
+        <v>20</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
+      <c r="C24" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A26:D26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2391,120 +2448,120 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>32</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B7" s="9" t="s">
         <v>32</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B11" s="9" t="s">
         <v>32</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>38</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -2535,137 +2592,137 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2692,83 +2749,83 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
     </row>
     <row r="11" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
@@ -2799,13 +2856,13 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>3</v>
@@ -2813,50 +2870,50 @@
     </row>
     <row r="4" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2883,14 +2940,14 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2911,10 +2968,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2922,10 +2979,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2933,10 +2990,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2944,10 +3001,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2955,15 +3012,15 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -2984,7 +3041,7 @@
   <sheetPr>
     <tabColor rgb="FFEA580C"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -2994,85 +3051,96 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>200</v>
+        <v>203</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
-        <v>207</v>
-      </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+        <v>209</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>214</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>